<commit_message>
fix: apply independent audit findings to customs rows and ND102 tax corrections
- Customs: ND128 Dieu 24.1 amounts ('tu X den Y dong'), confiscation attached for ND169 Dieu 18 / ND128 Dieu 17 (with the
  'tru' exclusion), tax-evasion condition (khoan 2), paragraphs after a point moved from the act text to notes,
  note truncated at a capitalised decree number
- Verification gate: tolerant amount pattern, row-set completeness against the extractor output
- Tax: status wording of rows replaced by ND102, general rules for ND102 transition and Dieu 43 exemption/reduction

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P9uqPmC9aiWESVacnFppTb
</commit_message>
<xml_diff>
--- a/outputs/penalty_catalog/penalty_catalog.xlsx
+++ b/outputs/penalty_catalog/penalty_catalog.xlsx
@@ -7217,7 +7217,7 @@
       </c>
       <c r="S91" s="4" t="inlineStr">
         <is>
-          <t>Đã được thay bằng quy định mới từ 16/01/2026 (chỉ áp dụng hành vi đã kết thúc trước ngày này)</t>
+          <t>Đã được NĐ102/2021 thay bằng quy định mới từ 01/01/2022 (chỉ áp dụng cho hành vi đã kết thúc trước ngày này)</t>
         </is>
       </c>
       <c r="T91" s="4" t="inlineStr">
@@ -10339,7 +10339,7 @@
       </c>
       <c r="S133" s="4" t="inlineStr">
         <is>
-          <t>Đã được thay bằng quy định mới từ 16/01/2026 (chỉ áp dụng hành vi đã kết thúc trước ngày này)</t>
+          <t>Đã được NĐ102/2021 thay bằng quy định mới từ 01/01/2022 (chỉ áp dụng cho hành vi đã kết thúc trước ngày này)</t>
         </is>
       </c>
       <c r="T133" s="4" t="inlineStr">
@@ -20810,7 +20810,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>Tiêu thụ hàng hóa đang chịu sự giám sát hải quan, trừ trường hợp quy định tại khoản 5 Điều này. Trường hợp vi phạm quy định tại điểm này mà tang vật vi phạm thuộc đối tượng không chịu thuế, miễn thuế, hàng hóa áp dụng thuế suất theo hạn ngạch thuế quan và không vi phạm quy định về chính sách quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo quy định tại điểm g khoản 1 Điều 15 Nghị định này</t>
+          <t>Tiêu thụ hàng hóa đang chịu sự giám sát hải quan, trừ trường hợp quy định tại khoản 5 Điều này</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr">
@@ -22090,7 +22090,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N293" s="2" t="inlineStr"/>
+      <c r="N293" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O293" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22161,7 +22165,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N294" s="2" t="inlineStr"/>
+      <c r="N294" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O294" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22232,7 +22240,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N295" s="2" t="inlineStr"/>
+      <c r="N295" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O295" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22303,7 +22315,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N296" s="2" t="inlineStr"/>
+      <c r="N296" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O296" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22374,7 +22390,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N297" s="2" t="inlineStr"/>
+      <c r="N297" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O297" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22445,7 +22465,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N298" s="2" t="inlineStr"/>
+      <c r="N298" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O298" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22516,7 +22540,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N299" s="2" t="inlineStr"/>
+      <c r="N299" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O299" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22587,7 +22615,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N300" s="2" t="inlineStr"/>
+      <c r="N300" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O300" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22658,7 +22690,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N301" s="2" t="inlineStr"/>
+      <c r="N301" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O301" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22729,7 +22765,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N302" s="2" t="inlineStr"/>
+      <c r="N302" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O302" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -22800,7 +22840,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N303" s="2" t="inlineStr"/>
+      <c r="N303" s="2" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O303" s="2" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -24130,7 +24174,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P319" s="2" t="inlineStr"/>
+      <c r="P319" s="2" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q319" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
@@ -24209,7 +24257,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P320" s="2" t="inlineStr"/>
+      <c r="P320" s="2" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q320" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
@@ -24288,7 +24340,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P321" s="2" t="inlineStr"/>
+      <c r="P321" s="2" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q321" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
@@ -24367,7 +24423,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P322" s="2" t="inlineStr"/>
+      <c r="P322" s="2" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q322" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
@@ -24446,7 +24506,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P323" s="2" t="inlineStr"/>
+      <c r="P323" s="2" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q323" s="2" t="inlineStr">
         <is>
           <t>2026-07-01</t>
@@ -32718,7 +32782,7 @@
       </c>
       <c r="G432" s="4" t="inlineStr">
         <is>
-          <t>Vi phạm quy định tại khoản 1 Điều này mà người khai hải quan tự phát hiện và khai bổ sung hồ sơ thuế sau khi có kết luận kiểm tra, thanh tra. Vi phạm quy định tại các điểm b, c, d khoản này mà cá nhân, tổ chức vi phạm không tự nguyện khắc phục hậu quả bằng cách nộp đủ số tiền thuế phải nộp trước thời điểm lập biên bản vi phạm hành chính thì xử phạt theo quy định tại điểm c khoản 1 Điều 14 Nghị định này</t>
+          <t>Vi phạm quy định tại khoản 1 Điều này mà người khai hải quan tự phát hiện và khai bổ sung hồ sơ thuế sau khi có kết luận kiểm tra, thanh tra</t>
         </is>
       </c>
       <c r="H432" s="4" t="inlineStr">
@@ -36806,7 +36870,7 @@
       </c>
       <c r="G484" s="4" t="inlineStr">
         <is>
-          <t>Tiêu thụ hàng hóa đang chịu sự giám sát hải quan, trừ trường hợp quy định tại khoản 5 Điều này. Trường hợp vi phạm quy định tại điểm này mà tang vật vi phạm thuộc đối tượng không chịu thuế, miễn thuế, xét miễn thuế, hàng hóa áp dụng thuế suất theo hạn ngạch thuế quan và không vi phạm quy định về chính sách quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo quy định tại điểm g khoản 1 Điều 14 Nghị định này</t>
+          <t>Tiêu thụ hàng hóa đang chịu sự giám sát hải quan, trừ trường hợp quy định tại khoản 5 Điều này</t>
         </is>
       </c>
       <c r="H484" s="4" t="inlineStr">
@@ -38154,7 +38218,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N501" s="4" t="inlineStr"/>
+      <c r="N501" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O501" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38229,7 +38297,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N502" s="4" t="inlineStr"/>
+      <c r="N502" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O502" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38304,7 +38376,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N503" s="4" t="inlineStr"/>
+      <c r="N503" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O503" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38379,7 +38455,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N504" s="4" t="inlineStr"/>
+      <c r="N504" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O504" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38454,7 +38534,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N505" s="4" t="inlineStr"/>
+      <c r="N505" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O505" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38529,7 +38613,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N506" s="4" t="inlineStr"/>
+      <c r="N506" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O506" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38604,7 +38692,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N507" s="4" t="inlineStr"/>
+      <c r="N507" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O507" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38679,7 +38771,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N508" s="4" t="inlineStr"/>
+      <c r="N508" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O508" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38754,7 +38850,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N509" s="4" t="inlineStr"/>
+      <c r="N509" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O509" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38829,7 +38929,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N510" s="4" t="inlineStr"/>
+      <c r="N510" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O510" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -38904,7 +39008,11 @@
           <t>Phạt 01 lần số tiền thuế trốn trong trường hợp không có tình tiết tăng nặng; Trường hợp có tình tiết tăng nặng thì mỗi tình tiết tăng nặng mức phạt tăng lên 0,2 lần nhưng không vượt quá 03 lần số tiền thuế trốn</t>
         </is>
       </c>
-      <c r="N511" s="4" t="inlineStr"/>
+      <c r="N511" s="4" t="inlineStr">
+        <is>
+          <t>Người nộp thuế có hành vi vi phạm quy định tại khoản 1 Điều này mà không bị truy cứu trách nhiệm hình sự thì bị phạt tiền như sau</t>
+        </is>
+      </c>
       <c r="O511" s="4" t="inlineStr">
         <is>
           <t>Buộc nộp đủ số tiền thuế trốn đối với hành vi vi phạm quy định tại Điều này</t>
@@ -39950,7 +40058,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P523" s="4" t="inlineStr"/>
+      <c r="P523" s="4" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q523" s="4" t="inlineStr">
         <is>
           <t>2020-12-10</t>
@@ -40033,7 +40145,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P524" s="4" t="inlineStr"/>
+      <c r="P524" s="4" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q524" s="4" t="inlineStr">
         <is>
           <t>2020-12-10</t>
@@ -40116,7 +40232,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P525" s="4" t="inlineStr"/>
+      <c r="P525" s="4" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q525" s="4" t="inlineStr">
         <is>
           <t>2020-12-10</t>
@@ -40199,7 +40319,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P526" s="4" t="inlineStr"/>
+      <c r="P526" s="4" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q526" s="4" t="inlineStr">
         <is>
           <t>2020-12-10</t>
@@ -40282,7 +40406,11 @@
           <t>Buộc tiêu hủy tang vật vi phạm hành chính là hàng hóa, vật phẩm gây hại cho sức khỏe con người, vật nuôi, cây trồng và môi trường, văn hóa phẩm có nội dung độc hại đối với hành vi vi phạm quy định tại Điều này | Buộc nộp lại số tiền bằng trị giá tang vật đã bị tiêu thụ, tẩu tán, tiêu hủy trái quy định của pháp luật đối với hành vi vi phạm quy định tại Điều này</t>
         </is>
       </c>
-      <c r="P527" s="4" t="inlineStr"/>
+      <c r="P527" s="4" t="inlineStr">
+        <is>
+          <t>Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+        </is>
+      </c>
       <c r="Q527" s="4" t="inlineStr">
         <is>
           <t>2020-12-10</t>
@@ -44096,18 +44224,22 @@
       </c>
       <c r="H575" s="4" t="inlineStr">
         <is>
-          <t>Phạt theo tỷ lệ</t>
-        </is>
-      </c>
-      <c r="I575" s="5" t="n"/>
-      <c r="J575" s="5" t="n"/>
-      <c r="K575" s="5" t="n"/>
-      <c r="L575" s="5" t="n"/>
-      <c r="M575" s="4" t="inlineStr">
-        <is>
-          <t>Phạt tiền từ 1.000.000 đến 3.000.000 đồng</t>
-        </is>
-      </c>
+          <t>Phạt tiền (khung)</t>
+        </is>
+      </c>
+      <c r="I575" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J575" s="5" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="K575" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="L575" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="M575" s="4" t="inlineStr"/>
       <c r="N575" s="4" t="inlineStr"/>
       <c r="O575" s="4" t="inlineStr"/>
       <c r="P575" s="4" t="inlineStr"/>
@@ -44167,18 +44299,22 @@
       </c>
       <c r="H576" s="4" t="inlineStr">
         <is>
-          <t>Phạt theo tỷ lệ</t>
-        </is>
-      </c>
-      <c r="I576" s="5" t="n"/>
-      <c r="J576" s="5" t="n"/>
-      <c r="K576" s="5" t="n"/>
-      <c r="L576" s="5" t="n"/>
-      <c r="M576" s="4" t="inlineStr">
-        <is>
-          <t>Phạt tiền từ 1.000.000 đến 3.000.000 đồng</t>
-        </is>
-      </c>
+          <t>Phạt tiền (khung)</t>
+        </is>
+      </c>
+      <c r="I576" s="5" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J576" s="5" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="K576" s="5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="L576" s="5" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="M576" s="4" t="inlineStr"/>
       <c r="N576" s="4" t="inlineStr"/>
       <c r="O576" s="4" t="inlineStr"/>
       <c r="P576" s="4" t="inlineStr"/>
@@ -44855,7 +44991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -45075,7 +45211,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Hóa đơn: 01 năm với hành vi trước 01/01/2022; 02 năm từ 01/01/2022 (Điều 1.1 NĐ102/2021). Danh sách hành vi 'đang thực hiện' được NĐ310 sửa tại Điều 8.1. Thủ tục thuế: 02 năm. Trốn thuế (chưa đến mức hình sự) và khai sai dẫn đến thiếu thuế: 05 năm.</t>
+          <t>Hóa đơn: 01 năm với hành vi trước 01/01/2022; 02 năm từ 01/01/2022 (Điều 1.1 NĐ102/2021). Danh sách hành vi 'đang thực hiện' được NĐ310 sửa tại Điều 8.1. Thủ tục thuế: 02 năm. Trốn thuế (chưa đến mức hình sự) và khai sai dẫn đến thiếu thuế: 05 năm. Cách chia 01 năm / 02 năm theo ngày hành vi là cách hiểu của bảng (NĐ102 Điều 7.2 chỉ cho áp dụng quy định mới đối với hành vi cũ khi nhẹ hơn). NĐ102 Điều 6.1.b bãi bỏ khoản 3 Điều 8 NĐ125 (quy định riêng về hồ sơ do cơ quan tố tụng hình sự chuyển đến).</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -45092,7 +45228,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>NĐ125 hiệu lực 05/12/2020. NĐ102/2021 (sửa NĐ125) hiệu lực 01/01/2022. NĐ310 hiệu lực 16/01/2026. Hành vi đã kết thúc trước 16/01/2026: áp dụng văn bản có hiệu lực tại thời điểm vi phạm. Hành vi đang thực hiện trước ngày này và bị phát hiện sau ngày này: áp dụng NĐ310.</t>
+          <t>NĐ125 hiệu lực 05/12/2020. NĐ102/2021 (sửa NĐ125) hiệu lực 01/01/2022. NĐ310 hiệu lực 16/01/2026. Hành vi đã kết thúc trước 16/01/2026: áp dụng văn bản có hiệu lực tại thời điểm vi phạm. Hành vi đang thực hiện trước ngày này và bị phát hiện sau ngày này: áp dụng NĐ310. Với NĐ102/2021 (Điều 7): hành vi xảy ra trước 01/01/2022 bị phát hiện sau đó thì áp dụng NĐ102 nếu NĐ102 không quy định trách nhiệm pháp lý hoặc quy định nhẹ hơn; quyết định xử phạt đã ban hành mà còn khiếu nại: giải quyết theo nghị định có hiệu lực tại thời điểm hành vi; hồ sơ đề nghị miễn tiền phạt tiếp nhận trước 01/01/2022: theo NĐ125 gốc.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -45104,134 +45240,151 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Chưa nằm trong bảng này</t>
+          <t>Miễn, giảm tiền phạt (thuế, hóa đơn)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Tiền chậm nộp tiền thuế (tỷ lệ theo Luật Quản lý thuế - văn bản chưa được cung cấp, bảng này không nêu tỷ lệ); truy thu thuế; vi phạm hải quan, bảo hiểm xã hội, lao động; các nghị định xử phạt chuyên ngành khác.</t>
+          <t>Điều 43 NĐ125 do NĐ102 thay thế (từ 01/01/2022): thực hiện theo Điều 77 Luật Xử lý vi phạm hành chính. Mức miễn, giảm tối đa bằng số tiền phạt trong quyết định xử phạt và không quá giá trị tài sản, hàng hóa bị thiệt hại sau khi trừ giá trị được bảo hiểm, bồi thường (bất khả kháng cần hồ sơ chứng minh thiệt hại). Không miễn, giảm nếu đã thi hành xong quyết định xử phạt. Được miễn, giảm tiền phạt thì được miễn, giảm tiền chậm nộp tiền phạt tương ứng. Miễn, giảm không đúng bị hủy hoặc điều chỉnh, thu lại tiền phạt và tính tiền chậm nộp.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Điều 43 NĐ125 (thay thế bởi Điều 1.6 NĐ102/2021)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: văn bản áp dụng và quan hệ với NĐ125</t>
+          <t>Chưa nằm trong bảng này</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>NĐ 169/2026/NĐ-CP (hiệu lực 01/07/2026) thay thế NĐ 128/2020/NĐ-CP và Điều 2 NĐ 102/2021/NĐ-CP (Điều 38 NĐ169). NĐ125 KHÔNG áp dụng cho vi phạm về thuế đối với hàng xuất nhập khẩu do cơ quan hải quan quản lý thu (Điều 1.1 NĐ125): thuế xuất nhập khẩu dùng nghị định hải quan, không cộng với Điều 16, 17 NĐ125. NĐ 127/2013 (VBHN 10/2016) áp dụng cho hành vi trước 10/12/2020, nhưng thời hiệu tối đa 05 năm (Điều 3 VBHN) nên đã hết từ 10/12/2025; bảng này không gồm văn bản đó.</t>
+          <t>Tiền chậm nộp tiền thuế (tỷ lệ theo Luật Quản lý thuế - văn bản chưa được cung cấp, bảng này không nêu tỷ lệ); truy thu thuế; vi phạm hải quan, bảo hiểm xã hội, lao động; các nghị định xử phạt chuyên ngành khác.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Điều 38 NĐ169; Điều 1.1 NĐ125; Điều 35 NĐ128; Điều 3 VBHN 10/2016</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: chuyển tiếp 01/07/2026</t>
+          <t>Hải quan: văn bản áp dụng và quan hệ với NĐ125</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Hành vi xảy ra và kết thúc trước 01/07/2026 nhưng bị phát hiện hoặc xem xét xử phạt từ 01/07/2026: áp dụng NĐ169 nếu NĐ169 không quy định trách nhiệm pháp lý hoặc quy định nhẹ hơn; nếu NĐ169 nặng hơn thì áp dụng NĐ128 (+ NĐ102). Bảng chọn bản theo ngày hành vi kết thúc; với hành vi trước 01/07/2026 nên xem cả hai bản và chọn bản nhẹ hơn.</t>
+          <t>NĐ 169/2026/NĐ-CP (hiệu lực 01/07/2026) thay thế NĐ 128/2020/NĐ-CP và Điều 2 NĐ 102/2021/NĐ-CP (Điều 38 NĐ169). NĐ125 KHÔNG áp dụng cho vi phạm về thuế đối với hàng xuất nhập khẩu do cơ quan hải quan quản lý thu (Điều 1.1 NĐ125): thuế xuất nhập khẩu dùng nghị định hải quan, không cộng với Điều 16, 17 NĐ125. NĐ 127/2013 (VBHN 10/2016) áp dụng cho hành vi trước 10/12/2020, nhưng thời hiệu tối đa 05 năm (Điều 3 VBHN) nên đã hết từ 10/12/2025; bảng này không gồm văn bản đó.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Điều 39 NĐ169; Điều 36 NĐ128; Điều 7 NĐ102/2021</t>
+          <t>Điều 38 NĐ169; Điều 1.1 NĐ125; Điều 35 NĐ128; Điều 3 VBHN 10/2016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: mức phạt cá nhân so với tổ chức</t>
+          <t>Hải quan: chuyển tiếp 01/07/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Khung tiền ở Chương II là mức cho TỔ CHỨC; cá nhân bằng 1/2, TRỪ: (1) hành vi xuất cảnh, nhập cảnh (Điều 11 NĐ169; Điều 10 NĐ128) - khung đã là mức của cá nhân; (2) hành vi về quản lý thuế (Điều 10, 15 NĐ169; Điều 9, 14 NĐ128) - cùng mức cho cá nhân và tổ chức. Hộ kinh doanh, hộ gia đình, cộng đồng dân cư áp dụng như cá nhân.</t>
+          <t>Hành vi xảy ra và kết thúc trước 01/07/2026 nhưng bị phát hiện hoặc xem xét xử phạt từ 01/07/2026: áp dụng NĐ169 nếu NĐ169 không quy định trách nhiệm pháp lý hoặc quy định nhẹ hơn; nếu NĐ169 nặng hơn thì áp dụng NĐ128 (+ NĐ102). Bảng chọn bản theo ngày hành vi kết thúc; với hành vi trước 01/07/2026 nên xem cả hai bản và chọn bản nhẹ hơn.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Điều 6.3 NĐ169; Điều 5.3 NĐ128</t>
+          <t>Điều 39 NĐ169; Điều 36 NĐ128; Điều 7 NĐ102/2021</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: mức cụ thể trong khung</t>
+          <t>Hải quan: mức phạt cá nhân so với tổ chức</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Mức phạt cụ thể = mức trung bình của khung. NĐ169 (từ 01/07/2026): 1 tình tiết giảm nhẹ giảm 10%, từ 2 tình tiết giảm nhẹ áp mức tối thiểu; 1 tình tiết tăng nặng tăng 10%, từ 2 tình tiết tăng nặng áp mức tối đa; một tình tiết giảm nhẹ bù trừ một tình tiết tăng nặng. Áp dụng cho Điều 8, 9, 11-14, 16-25 và khoản 1, 2, 4 Điều 26. NĐ128 (+ NĐ102 từ 01/01/2022): mỗi tình tiết ±10% mức trung bình, không vượt khung; áp dụng cho Điều 7, 8, 10-13, 15-24 và khoản 1, 3, 4 Điều 25. Tình tiết giảm nhẹ riêng của hải quan: tang vật có trị giá không quá 50% mức phạt tối thiểu của khung.</t>
+          <t>Khung tiền ở Chương II là mức cho TỔ CHỨC; cá nhân bằng 1/2, TRỪ: (1) hành vi xuất cảnh, nhập cảnh (Điều 11 NĐ169; Điều 10 NĐ128) - khung đã là mức của cá nhân; (2) hành vi về quản lý thuế (Điều 10, 15 NĐ169; Điều 9, 14 NĐ128) - cùng mức cho cá nhân và tổ chức. Hộ kinh doanh, hộ gia đình, cộng đồng dân cư áp dụng như cá nhân.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Điều 4, Điều 6.3.đ, e NĐ169; Điều 3, Điều 5.3.đ, e NĐ128 (NĐ102/2021 Điều 2.3)</t>
+          <t>Điều 6.3 NĐ169; Điều 5.3 NĐ128</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: trốn thuế và khai sai thuế</t>
+          <t>Hải quan: mức cụ thể trong khung</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Trốn thuế (Điều 15 NĐ169; Điều 14 NĐ128): phạt 01 lần số thuế trốn; mỗi tình tiết tăng nặng +0,2 lần, tối đa 03 lần (khác Điều 17 NĐ125). Khai sai dẫn đến thiếu thuế (Điều 10 NĐ169; Điều 9 NĐ128): phạt 10% số thuế khai thiếu nếu tự phát hiện, khai bổ sung muộn; 20% nếu hải quan phát hiện; chỉ xử phạt khi số thuế chênh lệch từ 500.000 đ/tờ khai (cá nhân), 2.000.000 đ/tờ khai (tổ chức). Không xử phạt nếu khai bổ sung trong hạn (60 ngày kể từ ngày thông quan và trước quyết định kiểm tra, thanh tra) - Điều 7.2.a NĐ169.</t>
+          <t>Mức phạt cụ thể = mức trung bình của khung. NĐ169 (từ 01/07/2026): 1 tình tiết giảm nhẹ giảm 10%, từ 2 tình tiết giảm nhẹ áp mức tối thiểu; 1 tình tiết tăng nặng tăng 10%, từ 2 tình tiết tăng nặng áp mức tối đa; một tình tiết giảm nhẹ bù trừ một tình tiết tăng nặng. Áp dụng cho Điều 8, 9, 11-14, 16-25 và khoản 1, 2, 4 Điều 26. NĐ128 (+ NĐ102 từ 01/01/2022): mỗi tình tiết ±10% mức trung bình, không vượt khung; áp dụng cho Điều 7, 8, 10-13, 15-24 và khoản 1, 3, 4 Điều 25. Tình tiết giảm nhẹ riêng của hải quan: tang vật có trị giá không quá 50% mức phạt tối thiểu của khung.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Điều 10, 15, 7.2.a NĐ169; Điều 9, 14 NĐ128</t>
+          <t>Điều 4, Điều 6.3.đ, e NĐ169; Điều 3, Điều 5.3.đ, e NĐ128 (NĐ102/2021 Điều 2.3)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Hải quan: thời hiệu</t>
+          <t>Hải quan: trốn thuế và khai sai thuế</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Thuế (trốn thuế chưa đến mức hình sự, khai sai dẫn đến thiếu thuế): 05 năm. Hành vi khác: 02 năm. Quá thời hiệu vẫn phải nộp đủ thuế thiếu, thuế trốn và tiền chậm nộp trong 10 năm trở về trước kể từ ngày phát hiện. Hồ sơ do cơ quan tố tụng chuyển đến: thời hiệu kéo dài thêm 01 năm (NĐ169).</t>
+          <t>Trốn thuế (Điều 15 NĐ169; Điều 14 NĐ128): phạt 01 lần số thuế trốn; mỗi tình tiết tăng nặng +0,2 lần, tối đa 03 lần (khác Điều 17 NĐ125). Khai sai dẫn đến thiếu thuế (Điều 10 NĐ169; Điều 9 NĐ128): phạt 10% số thuế khai thiếu nếu tự phát hiện, khai bổ sung muộn; 20% nếu hải quan phát hiện; chỉ xử phạt khi số thuế chênh lệch từ 500.000 đ/tờ khai (cá nhân), 2.000.000 đ/tờ khai (tổ chức). Không xử phạt nếu khai bổ sung trong hạn (60 ngày kể từ ngày thông quan và trước quyết định kiểm tra, thanh tra) - Điều 7.2.a NĐ169.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Điều 5 NĐ169; Điều 4 NĐ128</t>
+          <t>Điều 10, 15, 7.2.a NĐ169; Điều 9, 14 NĐ128</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>Hải quan: thời hiệu</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Thuế (trốn thuế chưa đến mức hình sự, khai sai dẫn đến thiếu thuế): 05 năm. Hành vi khác: 02 năm. Quá thời hiệu vẫn phải nộp đủ thuế thiếu, thuế trốn và tiền chậm nộp trong 10 năm trở về trước kể từ ngày phát hiện. Hồ sơ do cơ quan tố tụng chuyển đến: thời hiệu kéo dài thêm 01 năm (NĐ169).</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Điều 5 NĐ169; Điều 4 NĐ128</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>Hải quan: vi phạm nhiều lần, cảnh cáo, hình sự</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Vi phạm nhiều lần: xử phạt từng hành vi, trừ một số hành vi trên nhiều tờ khai/chứng từ được phát hiện cùng lúc thì phạt một lần và áp dụng tình tiết tăng nặng (Điều 3.1 NĐ169; Điều 2a NĐ128). Cảnh cáo chỉ áp dụng cho cá nhân từ 14 đến dưới 16 tuổi. Hành vi đến mức truy cứu trách nhiệm hình sự không thuộc bảng này (Điều 3.3 NĐ169: ngưỡng 100 triệu đồng với cá nhân, 200 triệu đồng với tổ chức theo trị giá tang vật hoặc số thuế trốn).</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Điều 3, Điều 6.2 NĐ169; Điều 2a, Điều 5.2 NĐ128</t>
         </is>
@@ -45248,7 +45401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -45464,7 +45617,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Khoản 4: Vận chuyển ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “Vận chuyển lâm sản trái pháp luật” quy định tại Điều 25 Nghị định số 146/2026/NĐ-CP ngày 06 tháng 5 năm 2026 của Chính phủ quy định xử phạt vi phạm hành chính trong lĩnh vực lâm nghiệp; xuất khẩu, nhập khẩu ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “tàng trữ, mua bán, xuất khẩu, nhập khẩu, chế biến lâm sản trái pháp luật” quy định tại Điều 26 Nghị định số</t>
+          <t>Khoản 4: Vận chuyển ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “Vận chuyển lâm sản trái pháp luật” quy định tại Điều 25 Nghị định số 146/2026/NĐ-CP ngày 06 tháng 5 năm 2026 của Chính phủ quy định xử phạt vi phạm hành chính trong lĩnh vực lâm nghiệp; xuất khẩu, nhập khẩu ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “tàng trữ, mua bán, xuất khẩu, nhập khẩu, chế biến lâm sản trái pháp luật” quy định tại Điều 26 Nghị định số 146/2026/NĐ-CP</t>
         </is>
       </c>
     </row>
@@ -45475,11 +45628,11 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Hình thức xử phạt bổ sung (khoản 2): Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
+          <t>Khoản 1: Các hành vi vi phạm quy định về xuất khẩu, nhập khẩu hàng hóa theo điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật gồm: Xuất khẩu, nhập khẩu hàng hóa không đáp ứng điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật; Xuất khẩu, nhập khẩu hàng hóa phải kiểm tra chuyên ngành mà không có thông báo kết quả kiểm tra chuyên ngành theo quy định của pháp luật</t>
         </is>
       </c>
     </row>
@@ -45494,7 +45647,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Khoản 1: Các hành vi vi phạm quy định về xuất khẩu, nhập khẩu hàng hóa theo điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật gồm: Xuất khẩu, nhập khẩu hàng hóa không đáp ứng điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật; Xuất khẩu, nhập khẩu hàng hóa phải kiểm tra chuyên ngành mà không có thông báo kết quả kiểm tra chuyên ngành theo quy định của pháp luật</t>
+          <t>Khoản 2: Nhập khẩu hàng hóa không có chứng từ chứng nhận xuất xứ hàng hóa mà theo quy định phải có chứng từ chứng nhận xuất xứ hàng hóa để xác định hàng hóa không có xuất xứ từ các nước có nguy cơ gây hại đến an toàn xã hội, sức khỏe của cộng đồng hoặc vệ sinh môi trường cần được kiểm soát</t>
         </is>
       </c>
     </row>
@@ -45509,22 +45662,22 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Khoản 2: Nhập khẩu hàng hóa không có chứng từ chứng nhận xuất xứ hàng hóa mà theo quy định phải có chứng từ chứng nhận xuất xứ hàng hóa để xác định hàng hóa không có xuất xứ từ các nước có nguy cơ gây hại đến an toàn xã hội, sức khỏe của cộng đồng hoặc vệ sinh môi trường cần được kiểm soát</t>
+          <t>Khoản 7: Giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật nêu tại Điều này là giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật quy định tại Luật Quản lý ngoại thương số 05/2017/QH14 và các văn bản quy phạm pháp luật khác có quy định về giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật đối với hàng hóa xuất khẩu, nhập khẩu; điều kiện về chủ thể kinh doanh mà thương nhân phải đáp ứng khi thực hiện hoạt động xuất khẩu, nhập khẩu</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>NĐ 169/2026</t>
+          <t>NĐ 128/2020</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Khoản 7: Giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật nêu tại Điều này là giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật quy định tại Luật Quản lý ngoại thương số 05/2017/QH14 và các văn bản quy phạm pháp luật khác có quy định về giấy phép, điều kiện, tiêu chuẩn kỹ thuật, quy chuẩn kỹ thuật đối với hàng hóa xuất khẩu, nhập khẩu; điều kiện về chủ thể kinh doanh mà thương nhân phải đáp ứng khi thực hiện hoạt động xuất khẩu, nhập khẩu</t>
+          <t>Khoản 7: Vi phạm quy định tại điểm b khoản 1, khoản 3, khoản 5 Điều này dẫn đến thiếu số tiền thuế phải nộp hoặc tăng số tiền thuế được miễn, giảm, hoàn, không thu hoặc trốn thuế hoặc vi phạm quy định pháp luật về quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo các Điều 9, 14, 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45539,7 +45692,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Khoản 7: Vi phạm quy định tại điểm b khoản 1, khoản 3, khoản 5 Điều này dẫn đến thiếu số tiền thuế phải nộp hoặc tăng số tiền thuế được miễn, giảm, hoàn, không thu hoặc trốn thuế hoặc vi phạm quy định pháp luật về quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo các Điều 9, 14, 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
+          <t>Khoản 8: Quy định tại Điều này không áp dụng đối với trường hợp vi phạm quy định tại khoản 8 Điều 11 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45550,11 +45703,11 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Khoản 8: Quy định tại Điều này không áp dụng đối với trường hợp vi phạm quy định tại khoản 8 Điều 11 Nghị định này</t>
+          <t>Khoản 1: Các hành vi khai sai dẫn đến thiếu số tiền thuế phải nộp hoặc tăng số tiền thuế được miễn, giảm, hoàn, không thu gồm: Khai sai về lượng, tên hàng, chủng loại, chất lượng, trị giá hải quan, mã số hàng hóa, thuế suất, mức thuế, xuất xứ, trừ quy định tại khoản 8 Điều 11, điểm b khoản 1 Điều 14 Nghị định này; Khai sai đối tượng không chịu thuế, đối tượng miễn thuế, hàng quản lý theo hạn ngạch thuế quan; Lập và khai không đúng các nội dung trong hồ sơ miễn thuế, hồ sơ xét miễn, giảm thuế, hoàn thuế, không thu thuế, hồ sơ xử lý tiền thuế, tiền phạt nộp thừa; Vi phạm quy định về quản lý nguyên liệu, vật tư, máy móc, thiết bị, sản phẩm gia công, sản xuất xuất khẩu, chế xuất dẫn đến hàng hóa thực tế tồn kho thiếu so với chứng từ kế toán, sổ kế toán, hồ sơ hải quan đối với hàng hóa xuất khẩu, nhập khẩu mà không thuộc trường hợp quy định tại các điểm d, đ, e và điểm g khoản 1 Điều 14 Nghị định này; Vi phạm quy định quản lý hàng hóa trong kho bảo thuế dẫn đến hàng hóa thực tế tồn kho thiếu so với chứng từ, sổ sách kế toán, hồ sơ hải quan đối với hàng hóa xuất khẩu, nhập khẩu mà không thuộc trường hợp quy định tại điểm g khoản 1 Điều 14 Nghị định này; Lập báo cáo quyết toán về lượng nguyên liệu, vật tư, linh kiện nhập khẩu đã sử dụng để sản xuất không đúng với thực tế sử dụng để sản xuất sản phẩm gia công, sản phẩm xuất khẩu; Khai báo hàng hóa nhập khẩu theo loại hình gia công, sản xuất xuất khẩu nhưng không có cơ sở sản xuất hàng gia công, cơ sở sản xuất hàng xuất khẩu trên lãnh thổ nước Cộng hòa xã hội chủ nghĩa Việt Nam; hoặc không có máy móc, thiết bị thuộc quyền sở hữu hoặc quyền sử dụng tại cơ sở sản xuất phù hợp với nguyên liệu, vật tư, linh kiện nhập khẩu để gia công, sản xuất hàng xuất khẩu</t>
         </is>
       </c>
     </row>
@@ -45569,7 +45722,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Khoản 1: Các hành vi khai sai dẫn đến thiếu số tiền thuế phải nộp hoặc tăng số tiền thuế được miễn, giảm, hoàn, không thu gồm: Khai sai về lượng, tên hàng, chủng loại, chất lượng, trị giá hải quan, mã số hàng hóa, thuế suất, mức thuế, xuất xứ, trừ quy định tại khoản 8 Điều 11, điểm b khoản 1 Điều 14 Nghị định này; Khai sai đối tượng không chịu thuế, đối tượng miễn thuế, hàng quản lý theo hạn ngạch thuế quan; Lập và khai không đúng các nội dung trong hồ sơ miễn thuế, hồ sơ xét miễn, giảm thuế, hoàn thuế, không thu thuế, hồ sơ xử lý tiền thuế, tiền phạt nộp thừa; Vi phạm quy định về quản lý nguyên liệu, vật tư, máy móc, thiết bị, sản phẩm gia công, sản xuất xuất khẩu, chế xuất dẫn đến hàng hóa thực tế tồn kho thiếu so với chứng từ kế toán, sổ kế toán, hồ sơ hải quan đối với hàng hóa xuất khẩu, nhập khẩu mà không thuộc trường hợp quy định tại các điểm d, đ, e và điểm g khoản 1 Điều 14 Nghị định này; Vi phạm quy định quản lý hàng hóa trong kho bảo thuế dẫn đến hàng hóa thực tế tồn kho thiếu so với chứng từ, sổ sách kế toán, hồ sơ hải quan đối với hàng hóa xuất khẩu, nhập khẩu mà không thuộc trường hợp quy định tại điểm g khoản 1 Điều 14 Nghị định này; Lập báo cáo quyết toán về lượng nguyên liệu, vật tư, linh kiện nhập khẩu đã sử dụng để sản xuất không đúng với thực tế sử dụng để sản xuất sản phẩm gia công, sản phẩm xuất khẩu; Khai báo hàng hóa nhập khẩu theo loại hình gia công, sản xuất xuất khẩu nhưng không có cơ sở sản xuất hàng gia công, cơ sở sản xuất hàng xuất khẩu trên lãnh thổ nước Cộng hòa xã hội chủ nghĩa Việt Nam; hoặc không có máy móc, thiết bị thuộc quyền sở hữu hoặc quyền sử dụng tại cơ sở sản xuất phù hợp với nguyên liệu, vật tư, linh kiện nhập khẩu để gia công, sản xuất hàng xuất khẩu</t>
+          <t>Khoản 5: Thực hiện xử phạt theo quy định tại các khoản 1, 2 và 3 Điều này chỉ áp dụng trong trường hợp số tiền thuế chênh lệch từ 500.000 đồng/tờ khai hải quan đối với vi phạm do cá nhân thực hiện, từ 2.000.000 đồng/tờ khai hải quan đối với vi phạm do tổ chức thực hiện</t>
         </is>
       </c>
     </row>
@@ -45584,7 +45737,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Khoản 5: Thực hiện xử phạt theo quy định tại các khoản 1, 2 và 3 Điều này chỉ áp dụng trong trường hợp số tiền thuế chênh lệch từ 500.000 đồng/tờ khai hải quan đối với vi phạm do cá nhân thực hiện, từ 2.000.000 đồng/tờ khai hải quan đối với vi phạm do tổ chức thực hiện</t>
+          <t>Khoản 6: Vi phạm quy định tại các khoản 1, 2 và 3 Điều này là hành vi trốn thuế thì xử phạt theo quy định tại Điều 14 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45599,7 +45752,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Khoản 6: Vi phạm quy định tại các khoản 1, 2 và 3 Điều này là hành vi trốn thuế thì xử phạt theo quy định tại Điều 14 Nghị định này</t>
+          <t>Khoản 7: Quy định tại Điều này không áp dụng đối với các trường hợp vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45610,11 +45763,11 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Khoản 7: Quy định tại Điều này không áp dụng đối với các trường hợp vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
+          <t>Khoản 6: Trị giá tang vật vi phạm tại Điều này là trị giá sau khi đã trừ đi trị giá ngoại tệ tiền mặt, đồng Việt Nam bằng tiền mặt, công cụ chuyển nhượng, vàng, kim loại quý khác, đá quý không phải khai hải quan theo quy định của pháp luật</t>
         </is>
       </c>
     </row>
@@ -45625,11 +45778,11 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Khoản 6: Trị giá tang vật vi phạm tại Điều này là trị giá sau khi đã trừ đi trị giá ngoại tệ tiền mặt, đồng Việt Nam bằng tiền mặt, công cụ chuyển nhượng, vàng, kim loại quý khác, đá quý không phải khai hải quan theo quy định của pháp luật</t>
+          <t>Khoản 11: Cá nhân, tổ chức có hành vi vi phạm quy định tại điểm a khoản 7 Điều này để trốn thuế thì bị xử phạt theo quy định tại Điều 14 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45640,11 +45793,11 @@
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Khoản 11: Cá nhân, tổ chức có hành vi vi phạm quy định tại điểm a khoản 7 Điều này để trốn thuế thì bị xử phạt theo quy định tại Điều 14 Nghị định này</t>
+          <t>Khoản 9: Cá nhân, tổ chức có hành vi vi phạm quy định tại điểm a khoản 4, khoản 5, khoản 6 Điều này mà hàng hóa đã bị tiêu thụ và vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này thì ngoài việc bị xử phạt theo điểm a khoản 4, khoản 5, khoản 6 Điều này còn bị xử phạt về hành vi tương ứng quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45655,11 +45808,11 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Khoản 9: Cá nhân, tổ chức có hành vi vi phạm quy định tại điểm a khoản 4, khoản 5, khoản 6 Điều này mà hàng hóa đã bị tiêu thụ và vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này thì ngoài việc bị xử phạt theo điểm a khoản 4, khoản 5, khoản 6 Điều này còn bị xử phạt về hành vi tương ứng quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
+          <t>Khoản 4: Quy định tại Điều này không áp dụng đối với các trường hợp vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45674,7 +45827,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Khoản 4: Quy định tại Điều này không áp dụng đối với các trường hợp vi phạm quy định tại các Điều 15, 16, 17, 18, 19, 20, 21, 22 Nghị định này</t>
+          <t>Khoản 5: Vi phạm quy định tại các điểm c, h khoản 1 Điều này mà không có chứng từ để khai bổ sung thì xử phạt theo quy định tại khoản 8 Điều 11 Nghị định này</t>
         </is>
       </c>
     </row>
@@ -45685,11 +45838,11 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Khoản 5: Vi phạm quy định tại các điểm c, h khoản 1 Điều này mà không có chứng từ để khai bổ sung thì xử phạt theo quy định tại khoản 8 Điều 11 Nghị định này</t>
+          <t>Khoản 2: Mang vào hoặc mang ra khỏi lãnh thổ nước Cộng hòa xã hội chủ nghĩa Việt Nam trái phép ma túy, vũ khí, pháo các loại thuộc danh mục hàng cấm xuất khẩu, cấm nhập khẩu hoặc tạm ngừng xuất khẩu, tạm ngừng nhập khẩu thì xử phạt theo quy định tại Nghị định số 167/2013/NĐ-CP ngày 12 tháng 11 năm 2013 của Chính phủ quy định xử phạt vi phạm hành chính trong lĩnh vực an ninh, trật tự, an toàn xã hội; phòng, chống tệ nạn xã hội; phòng cháy, chữa cháy; phòng, chống bạo lực gia đình</t>
         </is>
       </c>
     </row>
@@ -45704,37 +45857,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Khoản 2: Mang vào hoặc mang ra khỏi lãnh thổ nước Cộng hòa xã hội chủ nghĩa Việt Nam trái phép ma túy, vũ khí, pháo các loại thuộc danh mục hàng cấm xuất khẩu, cấm nhập khẩu hoặc tạm ngừng xuất khẩu, tạm ngừng nhập khẩu thì xử phạt theo quy định tại Nghị định số 167/2013/NĐ-CP ngày 12 tháng 11 năm 2013 của Chính phủ quy định xử phạt vi phạm hành chính trong lĩnh vực an ninh, trật tự, an toàn xã hội; phòng, chống tệ nạn xã hội; phòng cháy, chữa cháy; phòng, chống bạo lực gia đình</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>NĐ 128/2020</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
           <t>Khoản 3: Vận chuyển ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “Vận chuyển lâm sản trái pháp luật” quy định tại Điều 22 Nghị định số 35/2019/NĐ-CP ngày 25 tháng 4 năm 2019 của Chính phủ quy định xử phạt vi phạm hành chính trong lĩnh vực lâm nghiệp; xuất khẩu, nhập khẩu ngà voi, sừng tê giác thuộc loại cấm xuất khẩu, cấm nhập khẩu bị xử phạt về hành vi “mua bán lâm sản trái pháp luật” quy định tại Điều 23 Nghị định số 35/2019/NĐ-CP</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>NĐ 128/2020</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>Hình thức xử phạt bổ sung (khoản 2): Tịch thu tang vật vi phạm hành chính đối với hành vi vi phạm quy định tại Điều này, trừ tang vật vi phạm bị áp dụng biện pháp khắc phục hậu quả quy định tại điểm a khoản 3 Điều này</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: keep paragraph notes through the merge; assign them only to the points they name; fidelity check in the gate
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P9uqPmC9aiWESVacnFppTb
</commit_message>
<xml_diff>
--- a/outputs/penalty_catalog/penalty_catalog.xlsx
+++ b/outputs/penalty_catalog/penalty_catalog.xlsx
@@ -20850,7 +20850,11 @@
           <t>NĐ 169/2026</t>
         </is>
       </c>
-      <c r="U276" s="2" t="inlineStr"/>
+      <c r="U276" s="2" t="inlineStr">
+        <is>
+          <t>Trường hợp vi phạm quy định tại điểm này mà tang vật vi phạm thuộc đối tượng không chịu thuế, miễn thuế, hàng hóa áp dụng thuế suất theo hạn ngạch thuế quan và không vi phạm quy định về chính sách quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo quy định tại điểm g khoản 1 Điều 15 Nghị định này</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -32676,7 +32680,11 @@
           <t>NĐ 128/2020</t>
         </is>
       </c>
-      <c r="U430" s="4" t="inlineStr"/>
+      <c r="U430" s="4" t="inlineStr">
+        <is>
+          <t>Vi phạm quy định tại các điểm b, c, d khoản này mà cá nhân, tổ chức vi phạm không tự nguyện khắc phục hậu quả bằng cách nộp đủ số tiền thuế phải nộp trước thời điểm lập biên bản vi phạm hành chính thì xử phạt theo quy định tại điểm c khoản 1 Điều 14 Nghị định này</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="4" t="inlineStr">
@@ -32751,7 +32759,11 @@
           <t>NĐ 128/2020</t>
         </is>
       </c>
-      <c r="U431" s="4" t="inlineStr"/>
+      <c r="U431" s="4" t="inlineStr">
+        <is>
+          <t>Vi phạm quy định tại các điểm b, c, d khoản này mà cá nhân, tổ chức vi phạm không tự nguyện khắc phục hậu quả bằng cách nộp đủ số tiền thuế phải nộp trước thời điểm lập biên bản vi phạm hành chính thì xử phạt theo quy định tại điểm c khoản 1 Điều 14 Nghị định này</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="4" t="inlineStr">
@@ -32826,7 +32838,11 @@
           <t>NĐ 128/2020</t>
         </is>
       </c>
-      <c r="U432" s="4" t="inlineStr"/>
+      <c r="U432" s="4" t="inlineStr">
+        <is>
+          <t>Vi phạm quy định tại các điểm b, c, d khoản này mà cá nhân, tổ chức vi phạm không tự nguyện khắc phục hậu quả bằng cách nộp đủ số tiền thuế phải nộp trước thời điểm lập biên bản vi phạm hành chính thì xử phạt theo quy định tại điểm c khoản 1 Điều 14 Nghị định này</t>
+        </is>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="4" t="inlineStr">
@@ -36914,7 +36930,11 @@
           <t>NĐ 128/2020</t>
         </is>
       </c>
-      <c r="U484" s="4" t="inlineStr"/>
+      <c r="U484" s="4" t="inlineStr">
+        <is>
+          <t>Trường hợp vi phạm quy định tại điểm này mà tang vật vi phạm thuộc đối tượng không chịu thuế, miễn thuế, xét miễn thuế, hàng hóa áp dụng thuế suất theo hạn ngạch thuế quan và không vi phạm quy định về chính sách quản lý hàng hóa xuất khẩu, nhập khẩu thì xử phạt theo quy định tại điểm g khoản 1 Điều 14 Nghị định này</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" s="4" t="inlineStr">

</xml_diff>